<commit_message>
Card Labs 3 and 4 built in: board conditions, Knight/Cleric adjacency and "alone" cards
- CardCondition (Assets/Scripts/Cards/CardCondition.cs): board conditions asked live for cost
  discounts and entry bonuses; Card/CardData/CardViewer read them on every look, the bot scores
  them through Card.EntryDelta/EntryLive.
- New Knight and Cleric cards from Card Lab III (adjacency) and Card Lab IV (alone at distance 3),
  plus Chapel, Spring and Warhorn totems with their effect assets and prefabs.
- Equipment: Longsword and Steel Sword added, Long Lens and Sharpening Ring removed, icons from
  the 60 free icons pack.
- CardSheet tooling learns the condition columns; baselines and design CSVs re-synced.
- balance-lab skill and labkit updates (ratings, cleanup, report); bot profile retunes.
- com.unity.ads removed from the manifest.
- Docs: CardLab3/4 handoffs, BotStrategy refresh, CLAUDE.md conditions section.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/EnemySheets.xlsx
+++ b/Docs/EnemySheets.xlsx
@@ -1254,7 +1254,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="2">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>6</v>
@@ -3013,7 +3013,7 @@
         <v>180</v>
       </c>
       <c r="B8" s="0">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -9493,7 +9493,7 @@
         <v>180</v>
       </c>
       <c r="B8" s="0">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -14179,7 +14179,7 @@
         <v>89</v>
       </c>
       <c r="E5" s="0">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F5" s="0">
         <v>1</v>
@@ -14241,7 +14241,7 @@
         <v>235</v>
       </c>
       <c r="E6" s="0">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F6" s="0">
         <v>1</v>
@@ -14489,7 +14489,7 @@
         <v>248</v>
       </c>
       <c r="E10" s="0">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F10" s="0">
         <v>1</v>
@@ -15047,7 +15047,7 @@
         <v>272</v>
       </c>
       <c r="E19" s="0">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F19" s="0">
         <v>1</v>
@@ -17930,7 +17930,7 @@
         <v>180</v>
       </c>
       <c r="B8" s="0">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -18740,7 +18740,7 @@
         <v>180</v>
       </c>
       <c r="B8" s="0">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">

</xml_diff>